<commit_message>
Update zone layouts knowledge base and backfill rule
- ZONE_LAYOUTS.md: current folder map, inventory and schema; how to
  build ZONE_MASTER from the KML (§6); updated open issues
- Client spec: backfilled zones set pit_available_to = effective_to

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/layouts/client/DEV_Korea Semiconductor Fab Activity Data_INFORMATION_20261021.xlsx
+++ b/layouts/client/DEV_Korea Semiconductor Fab Activity Data_INFORMATION_20261021.xlsx
@@ -3452,14 +3452,20 @@
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" spans="1:27" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" ht="105.0" customHeight="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="29" t="s">
         <v>77</v>
       </c>
       <c r="C22" s="30"/>
-      <c r="D22" s="103" t="s">
-        <v>318</v>
+      <c r="D22" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Every file is versioned the same way: a row is valid from pit_available_from until pit_available_to (NULL = current version). Key: (record_id, pit_available_from)
+- Real-world date: effective_from / effective_to (zones), effective_at (lineage), activity_at (foot-traffic and metrics)
+- Backtests: use rows where pit_available_from ≤ as-of date &lt; pit_available_to, or pit_available_to is NULL
+- Restatements: shipped rows are never edited; the row is closed with pit_available_to and a new row with the same record_id is added
+- Backfill: history before the first client release has pit_available_from = effective_from and pit_available_to = effective_to (zones), or pit_available_from = activity_date (foot-traffic)</t>
+        </is>
       </c>
       <c r="E22" s="90"/>
       <c r="F22" s="90"/>
@@ -3467,8 +3473,10 @@
       <c r="H22" s="58" t="s">
         <v>298</v>
       </c>
-      <c r="I22" s="58" t="s">
-        <v>319</v>
+      <c r="I22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PIT policy rewritten with Notion field names (effective_from/to, pit_available_from/to, record_id); adds backtest rule, restatement and backfill rules. Backfill rule now also sets pit_available_to = effective_to for zones.</t>
+        </is>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -4465,7 +4473,7 @@
       <c r="Z48" s="1"/>
       <c r="AA48" s="1"/>
     </row>
-    <row r="49" spans="1:27" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" ht="72.0" customHeight="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
       <c r="B49" s="42"/>
       <c r="C49" s="63" t="s">
@@ -4477,8 +4485,10 @@
       <c r="E49" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="F49" s="63" t="s">
-        <v>366</v>
+      <c r="F49" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date until which this specific record version was available to clients. NULL for the currently available version. For backfilled history (rows covering the period before the first client release), set equal to effective_to</t>
+        </is>
       </c>
       <c r="G49" s="63" t="s">
         <v>360</v>
@@ -4486,8 +4496,10 @@
       <c r="H49" s="58" t="s">
         <v>298</v>
       </c>
-      <c r="I49" s="58" t="s">
-        <v>361</v>
+      <c r="I49" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New field added per Notion FT_LIST_ZONE schema. Backfill rule added: pit_available_to = effective_to.</t>
+        </is>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>

</xml_diff>